<commit_message>
NeoEnergia pelos totais + reforma visual
</commit_message>
<xml_diff>
--- a/ACOES_SOCIAIS_levantamento.xlsx
+++ b/ACOES_SOCIAIS_levantamento.xlsx
@@ -788,6 +788,12 @@
           <t>012 - CEB</t>
         </is>
       </c>
+      <c r="B13" t="n">
+        <v>61</v>
+      </c>
+      <c r="C13" t="n">
+        <v>92</v>
+      </c>
       <c r="L13">
         <f>SUM(B13:K13)</f>
         <v/>
@@ -888,6 +894,9 @@
       <c r="C18" t="n">
         <v>1067</v>
       </c>
+      <c r="D18" t="n">
+        <v>1000</v>
+      </c>
       <c r="E18" t="n">
         <v>1727</v>
       </c>
@@ -1002,16 +1011,28 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>210</v>
+        <v>656</v>
       </c>
       <c r="C22" t="n">
-        <v>439</v>
+        <v>1015</v>
       </c>
       <c r="D22" t="n">
-        <v>361</v>
+        <v>1006</v>
       </c>
       <c r="E22" t="n">
-        <v>243</v>
+        <v>995</v>
+      </c>
+      <c r="G22" t="n">
+        <v>1779</v>
+      </c>
+      <c r="H22" t="n">
+        <v>446</v>
+      </c>
+      <c r="J22" t="n">
+        <v>651</v>
+      </c>
+      <c r="K22" t="n">
+        <v>867</v>
       </c>
       <c r="L22">
         <f>SUM(B22:K22)</f>
@@ -1058,7 +1079,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>57</v>
+        <v>91</v>
       </c>
       <c r="C26" t="n">
         <v>99</v>
@@ -1298,6 +1319,21 @@
         <is>
           <t>037 - CULTURA</t>
         </is>
+      </c>
+      <c r="C36" t="n">
+        <v>300</v>
+      </c>
+      <c r="D36" t="n">
+        <v>500</v>
+      </c>
+      <c r="G36" t="n">
+        <v>800</v>
+      </c>
+      <c r="H36" t="n">
+        <v>500</v>
+      </c>
+      <c r="J36" t="n">
+        <v>400</v>
       </c>
       <c r="L36">
         <f>SUM(B36:K36)</f>

</xml_diff>